<commit_message>
Parts list: tools are probably at the IYA Makerspace (counted as $0)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DUSU7jbUyc6QVB5XjyAbxC
</commit_message>
<xml_diff>
--- a/hardware/devboard/parts_list.xlsx
+++ b/hardware/devboard/parts_list.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="125">
   <si>
     <t xml:space="preserve">Parts WE buy</t>
   </si>
   <si>
-    <t xml:space="preserve">For 2 boards, with a spare where it helps. Prices are rough (Oct 2026). Tick "Bought?" as you go.</t>
+    <t xml:space="preserve">For 2 boards, with a spare where it helps. Prices are rough (Oct 2026). Tick "Bought?" as you go (for tools: once found at the IYA Makerspace).</t>
   </si>
   <si>
     <t xml:space="preserve">1. Goes ON the board (we solder these on)</t>
@@ -152,7 +152,7 @@
     <t xml:space="preserve">Solder the motor wires to it.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Tools (buy once)</t>
+    <t xml:space="preserve">3. Tools: probably at the IYA Makerspace (don't buy yet)</t>
   </si>
   <si>
     <t xml:space="preserve">Programmer</t>
@@ -164,6 +164,12 @@
     <t xml:space="preserve">Nordic nRF54L15 DK</t>
   </si>
   <si>
+    <t xml:space="preserve">IYA Makerspace (check first)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probably available at the IYA Makerspace. If not: ~$40 from Digi-Key / Mouser.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Debug cable</t>
   </si>
   <si>
@@ -173,10 +179,7 @@
     <t xml:space="preserve">10-pin 2x5, 1.27 mm cable</t>
   </si>
   <si>
-    <t xml:space="preserve">Adafruit / Digi-Key</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pull pin 7 on the board's debug header, or use an unkeyed cable.</t>
+    <t xml:space="preserve">Probably available at the IYA Makerspace. If not: ~$3. Pull pin 7 on the board's debug header, or use an unkeyed cable.</t>
   </si>
   <si>
     <t xml:space="preserve">Solder + flux</t>
@@ -188,7 +191,7 @@
     <t xml:space="preserve">Solder wire + no-clean flux</t>
   </si>
   <si>
-    <t xml:space="preserve">Amazon</t>
+    <t xml:space="preserve">Probably available at the IYA Makerspace. If not: ~$10.</t>
   </si>
   <si>
     <t xml:space="preserve">Heat-shrink tubing</t>
@@ -200,6 +203,9 @@
     <t xml:space="preserve">Small (1–2 mm) heat-shrink</t>
   </si>
   <si>
+    <t xml:space="preserve">Probably available at the IYA Makerspace. If not: ~$5.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Multimeter</t>
   </si>
   <si>
@@ -209,13 +215,13 @@
     <t xml:space="preserve">Any basic multimeter</t>
   </si>
   <si>
-    <t xml:space="preserve">Skip if someone has one.</t>
+    <t xml:space="preserve">Probably available at the IYA Makerspace. If not: ~$20.</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">Parts only. JLCPCB's board, assembly and shipping are separate (about $105–155 more).</t>
+    <t xml:space="preserve">Parts only; tools are counted as $0 (IYA Makerspace). JLCPCB's board, assembly and shipping are separate (about $105–155 more).</t>
   </si>
   <si>
     <t xml:space="preserve">JLCPCB makes the board and solders on everything else</t>
@@ -1193,7 +1199,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
         <v>44</v>
       </c>
@@ -1204,151 +1210,157 @@
         <v>46</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="E18" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="G18" s="10" t="n">
         <f aca="false">E18*F18</f>
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="H18" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="I18" s="7"/>
-    </row>
-    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I18" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>50</v>
-      </c>
       <c r="E19" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G19" s="10" t="n">
         <f aca="false">E19*F19</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H19" s="11" t="s">
         <v>16</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E20" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G20" s="10" t="n">
         <f aca="false">E20*F20</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H20" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="I20" s="7"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I20" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E21" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G21" s="10" t="n">
         <f aca="false">E21*F21</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H21" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="I21" s="7"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I21" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E22" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G22" s="10" t="n">
         <f aca="false">E22*F22</f>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H22" s="11" t="s">
         <v>16</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F24" s="12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G24" s="13" t="n">
         <f aca="false">SUMPRODUCT(E6:E23,F6:F23)</f>
-        <v>144.5</v>
+        <v>66.5</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1385,17 +1397,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1406,27 +1418,27 @@
         <v>4</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>1</v>
@@ -1434,16 +1446,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>1</v>
@@ -1451,16 +1463,16 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>1</v>
@@ -1468,16 +1480,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>1</v>
@@ -1485,16 +1497,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>1</v>
@@ -1502,16 +1514,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>1</v>
@@ -1519,16 +1531,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E12" s="7" t="n">
         <v>1</v>
@@ -1536,16 +1548,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E13" s="7" t="n">
         <v>1</v>
@@ -1553,16 +1565,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>1</v>
@@ -1570,16 +1582,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E15" s="7" t="n">
         <v>1</v>
@@ -1587,16 +1599,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E16" s="7" t="n">
         <v>1</v>
@@ -1604,16 +1616,16 @@
     </row>
     <row r="17" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E17" s="7" t="n">
         <v>24</v>
@@ -1621,22 +1633,22 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Parts list: drop the notes column
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DUSU7jbUyc6QVB5XjyAbxC
</commit_message>
<xml_diff>
--- a/hardware/devboard/parts_list.xlsx
+++ b/hardware/devboard/parts_list.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="105">
   <si>
     <t xml:space="preserve">JLCPCB order</t>
   </si>
@@ -68,7 +68,7 @@
     <t xml:space="preserve">LSM6DSV16BX</t>
   </si>
   <si>
-    <t xml:space="preserve">Motion + bone sensor (hears your voice through bone)</t>
+    <t xml:space="preserve">Motion + bone sensor</t>
   </si>
   <si>
     <t xml:space="preserve">U3</t>
@@ -188,7 +188,7 @@
     <t xml:space="preserve">Our order</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Goes ON the board (we solder these on)</t>
+    <t xml:space="preserve">On the board (we solder)</t>
   </si>
   <si>
     <t xml:space="preserve">Exact part number</t>
@@ -209,9 +209,6 @@
     <t xml:space="preserve">Bought?</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bluetooth module</t>
   </si>
   <si>
@@ -227,9 +224,6 @@
     <t xml:space="preserve">No</t>
   </si>
   <si>
-    <t xml:space="preserve">2 boards + 1 spare. NOT 453-00223, NOT a "-K1" kit.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Buttons</t>
   </si>
   <si>
@@ -242,10 +236,7 @@
     <t xml:space="preserve">Digi-Key</t>
   </si>
   <si>
-    <t xml:space="preserve">2 per board + 1 spare.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Plugs INTO the board</t>
+    <t xml:space="preserve">Plugs into the board</t>
   </si>
   <si>
     <t xml:space="preserve">Antenna</t>
@@ -260,9 +251,6 @@
     <t xml:space="preserve">Digi-Key / Mouser</t>
   </si>
   <si>
-    <t xml:space="preserve">Clicks onto the module.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Battery</t>
   </si>
   <si>
@@ -275,9 +263,6 @@
     <t xml:space="preserve">Adafruit</t>
   </si>
   <si>
-    <t xml:space="preserve">Don't cut the wire. Check + and − with a multimeter before plugging in.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Vibration motor</t>
   </si>
   <si>
@@ -287,9 +272,6 @@
     <t xml:space="preserve">Vybronics VG0832022D</t>
   </si>
   <si>
-    <t xml:space="preserve">The 022D (long wires), not the 013D. 2 + 1 spare.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Motor cable</t>
   </si>
   <si>
@@ -302,10 +284,7 @@
     <t xml:space="preserve">Amazon / Digi-Key</t>
   </si>
   <si>
-    <t xml:space="preserve">Solder the motor wires to it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Tools: probably at the IYA Makerspace (don't buy yet)</t>
+    <t xml:space="preserve">Tools (IYA Makerspace)</t>
   </si>
   <si>
     <t xml:space="preserve">Programmer</t>
@@ -317,10 +296,7 @@
     <t xml:space="preserve">Nordic nRF54L15 DK</t>
   </si>
   <si>
-    <t xml:space="preserve">IYA Makerspace (check first)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Probably available at the IYA Makerspace. If not: ~$40 from Digi-Key / Mouser.</t>
+    <t xml:space="preserve">IYA Makerspace</t>
   </si>
   <si>
     <t xml:space="preserve">Debug cable</t>
@@ -332,9 +308,6 @@
     <t xml:space="preserve">10-pin 2x5, 1.27 mm cable</t>
   </si>
   <si>
-    <t xml:space="preserve">Probably available at the IYA Makerspace. If not: ~$3. Pull pin 7 on the board's debug header, or use an unkeyed cable.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Solder + flux</t>
   </si>
   <si>
@@ -344,9 +317,6 @@
     <t xml:space="preserve">Solder wire + no-clean flux</t>
   </si>
   <si>
-    <t xml:space="preserve">Probably available at the IYA Makerspace. If not: ~$10.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Heat-shrink tubing</t>
   </si>
   <si>
@@ -356,9 +326,6 @@
     <t xml:space="preserve">Small (1–2 mm) heat-shrink</t>
   </si>
   <si>
-    <t xml:space="preserve">Probably available at the IYA Makerspace. If not: ~$5.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Multimeter</t>
   </si>
   <si>
@@ -366,9 +333,6 @@
   </si>
   <si>
     <t xml:space="preserve">Any basic multimeter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Probably available at the IYA Makerspace. If not: ~$20.</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -892,7 +856,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -1078,17 +1042,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1107,7 +1070,6 @@
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
@@ -1134,22 +1096,19 @@
       <c r="H4" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="I4" s="7" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>66</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>3</v>
@@ -1162,24 +1121,21 @@
         <v>18</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>70</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>72</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>5</v>
@@ -1192,15 +1148,12 @@
         <v>5</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -1209,7 +1162,6 @@
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
@@ -1236,22 +1188,19 @@
       <c r="H9" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="I9" s="7" t="s">
-        <v>62</v>
-      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>78</v>
       </c>
       <c r="E10" s="8" t="n">
         <v>2</v>
@@ -1264,24 +1213,21 @@
         <v>12</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="I10" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>79</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>83</v>
       </c>
       <c r="E11" s="8" t="n">
         <v>2</v>
@@ -1294,24 +1240,21 @@
         <v>12</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E12" s="8" t="n">
         <v>3</v>
@@ -1324,24 +1267,21 @@
         <v>15</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>88</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E13" s="8" t="n">
         <v>3</v>
@@ -1354,15 +1294,12 @@
         <v>4.5</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>93</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -1371,7 +1308,6 @@
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
@@ -1398,22 +1334,19 @@
       <c r="H16" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="I16" s="7" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="E17" s="8" t="n">
         <v>1</v>
@@ -1426,24 +1359,21 @@
         <v>0</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="I17" s="4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="E18" s="8" t="n">
         <v>1</v>
@@ -1456,24 +1386,21 @@
         <v>0</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>103</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="E19" s="8" t="n">
         <v>1</v>
@@ -1486,24 +1413,21 @@
         <v>0</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="I19" s="4" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="E20" s="8" t="n">
         <v>1</v>
@@ -1516,24 +1440,21 @@
         <v>0</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="I20" s="4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="E21" s="8" t="n">
         <v>1</v>
@@ -1546,15 +1467,12 @@
         <v>0</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>115</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F23" s="12" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="G23" s="13" t="n">
         <f aca="false">SUMPRODUCT(E5:E22,F5:F22)</f>

</xml_diff>

<commit_message>
Dev board: have JLCPCB fit the buttons and the radio module
Decided 2026-10-11: order 5 boards, all 5 fully assembled, nothing soldered by hand.

- SW1, SW2 (B3U-1000P, C231329, in stock) and U1 (453-00044R, C45868630, a JLCPCB
  pre-order part) are now FIT, so they appear in fab/bom.csv and fab/cpl.csv.
- README: order of steps (pre-order the module first), remark for U1 orientation,
  hand-soldering kept as the fallback.
- parts_list.xlsx: module and buttons moved to the JLCPCB tab.

Gerbers, schematic and PCB are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/devboard/parts_list.xlsx
+++ b/hardware/devboard/parts_list.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="14" min="1" max="1"/>
@@ -798,28 +798,78 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" ht="52.2" customHeight="1" s="15">
+    <row r="15" ht="15" customHeight="1" s="15">
       <c r="A15" s="18" t="inlineStr">
         <is>
+          <t>Bluetooth module (pre-order it first)</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>The brain + Bluetooth</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>C45868630</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="15">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Buttons</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>Power and calibrate buttons</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>SW1, SW2</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>C231329</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" ht="52.2" customHeight="1" s="15">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
           <t>Small parts</t>
         </is>
       </c>
-      <c r="B15" s="19" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>Resistors and capacitors (24 pieces)</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="C17" s="19" t="inlineStr">
         <is>
           <t>C1,C4,C11,C12,C17,C19, C2,C5,C6,C18,C20,C21, C3, C16, C8,C9,C10,C22, R1,R2, R3, R6, R7,R8</t>
         </is>
       </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>see bom.csv</t>
         </is>
       </c>
-      <c r="E15" s="19" t="n">
+      <c r="E17" s="19" t="n">
         <v>24</v>
       </c>
     </row>
@@ -836,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="14" min="1" max="1"/>
@@ -858,7 +908,7 @@
     <row r="3" ht="15" customHeight="1" s="15">
       <c r="A3" s="20" t="inlineStr">
         <is>
-          <t>On the board (we solder)</t>
+          <t>Plugs into the board</t>
         </is>
       </c>
       <c r="B3" s="21" t="n"/>
@@ -914,17 +964,17 @@
     <row r="5" ht="15" customHeight="1" s="15">
       <c r="A5" s="18" t="inlineStr">
         <is>
-          <t>Bluetooth module</t>
+          <t>Antenna</t>
         </is>
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>The brain + Bluetooth</t>
+          <t>Bluetooth signal</t>
         </is>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Ezurio BL54L15 453-00044R</t>
+          <t>Taoglas FXP830.24.0100B (MHF4 plug)</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -933,10 +983,10 @@
         </is>
       </c>
       <c r="E5" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" s="24" t="n">
-        <v>5.55</v>
+        <v>7.31</v>
       </c>
       <c r="G5" s="25">
         <f>E5*F5</f>
@@ -951,29 +1001,29 @@
     <row r="6" ht="15" customHeight="1" s="15">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Buttons</t>
+          <t>Battery</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Power and calibrate buttons</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>Omron (now Aratas) B3U-1000P</t>
+          <t>Adafruit #1570 (100 mAh LiPo)</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Digi-Key</t>
+          <t>Adafruit</t>
         </is>
       </c>
       <c r="E6" s="23" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F6" s="24" t="n">
-        <v>1.17</v>
+        <v>5.95</v>
       </c>
       <c r="G6" s="25">
         <f>E6*F6</f>
@@ -985,162 +1035,163 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="15">
-      <c r="A8" s="20" t="inlineStr">
-        <is>
-          <t>Plugs into the board</t>
-        </is>
-      </c>
-      <c r="B8" s="21" t="n"/>
-      <c r="C8" s="21" t="n"/>
-      <c r="D8" s="21" t="n"/>
-      <c r="E8" s="21" t="n"/>
-      <c r="F8" s="21" t="n"/>
-      <c r="G8" s="21" t="n"/>
-      <c r="H8" s="21" t="n"/>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="15">
-      <c r="A9" s="22" t="inlineStr">
+    <row r="7" ht="15" customHeight="1" s="15">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Vibration motor</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>The "tap"</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>Vybronics VG0832022D</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Digi-Key</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="24" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="G7" s="25">
+        <f>E7*F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="26.85" customHeight="1" s="15">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Motor cable</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Connects the motor to the board</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>JST SHR-02V-S housing + ASSHSSH28K102 lead, cut in half</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Digi-Key</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="24" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G8" s="25">
+        <f>E8*F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" s="15"/>
+    <row r="10" ht="15" customHeight="1" s="15">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>Tools (IYA Makerspace)</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="n"/>
+      <c r="C10" s="21" t="n"/>
+      <c r="D10" s="21" t="n"/>
+      <c r="E10" s="21" t="n"/>
+      <c r="F10" s="21" t="n"/>
+      <c r="G10" s="21" t="n"/>
+      <c r="H10" s="21" t="n"/>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="15">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="B9" s="22" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>What it is for</t>
         </is>
       </c>
-      <c r="C9" s="22" t="inlineStr">
+      <c r="C11" s="22" t="inlineStr">
         <is>
           <t>Exact part number</t>
         </is>
       </c>
-      <c r="D9" s="22" t="inlineStr">
+      <c r="D11" s="22" t="inlineStr">
         <is>
           <t>Buy from</t>
         </is>
       </c>
-      <c r="E9" s="22" t="inlineStr">
+      <c r="E11" s="22" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="F9" s="22" t="inlineStr">
+      <c r="F11" s="22" t="inlineStr">
         <is>
           <t>Price each</t>
         </is>
       </c>
-      <c r="G9" s="22" t="inlineStr">
+      <c r="G11" s="22" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="H9" s="22" t="inlineStr">
+      <c r="H11" s="22" t="inlineStr">
         <is>
           <t>Bought?</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="15">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Antenna</t>
-        </is>
-      </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>Bluetooth signal</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>Taoglas FXP830.24.0100B (MHF4 plug)</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>Digi-Key</t>
-        </is>
-      </c>
-      <c r="E10" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F10" s="24" t="n">
-        <v>7.31</v>
-      </c>
-      <c r="G10" s="25">
-        <f>E10*F10</f>
-        <v/>
-      </c>
-      <c r="H10" s="26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="15">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>Battery</t>
-        </is>
-      </c>
-      <c r="B11" s="19" t="inlineStr">
-        <is>
-          <t>Power</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="inlineStr">
-        <is>
-          <t>Adafruit #1570 (100 mAh LiPo)</t>
-        </is>
-      </c>
-      <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>Adafruit</t>
-        </is>
-      </c>
-      <c r="E11" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F11" s="24" t="n">
-        <v>5.95</v>
-      </c>
-      <c r="G11" s="25">
-        <f>E11*F11</f>
-        <v/>
-      </c>
-      <c r="H11" s="26" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="15">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>Vibration motor</t>
+          <t>Programmer</t>
         </is>
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>The "tap"</t>
+          <t>Puts our software on the board</t>
         </is>
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>Vybronics VG0832022D</t>
+          <t>Nordic nRF54L15-DK ($39 at Digi-Key if not borrowed)</t>
         </is>
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Digi-Key</t>
+          <t>IYA Makerspace</t>
         </is>
       </c>
       <c r="E12" s="23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>3.47</v>
+        <v>0</v>
       </c>
       <c r="G12" s="25">
         <f>E12*F12</f>
@@ -1152,32 +1203,32 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="26.85" customHeight="1" s="15">
+    <row r="13" ht="15" customHeight="1" s="15">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>Motor cable</t>
+          <t>Debug cable</t>
         </is>
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>Connects the motor to the board</t>
+          <t>Connects programmer to board</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>JST SHR-02V-S housing + ASSHSSH28K102 lead, cut in half</t>
+          <t>Samtec FFSD-05-D-02.00-01-N, 10-pin, 5 cm ($10.59 at Digi-Key)</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Digi-Key</t>
+          <t>IYA Makerspace</t>
         </is>
       </c>
       <c r="E13" s="23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="G13" s="25">
         <f>E13*F13</f>
@@ -1189,263 +1240,138 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="26.85" customHeight="1" s="15">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Solder + flux</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>To join the motor wires to the motor cable</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>Solder wire + no-clean flux</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>IYA Makerspace</t>
+        </is>
+      </c>
+      <c r="E14" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="25">
+        <f>E14*F14</f>
+        <v/>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
     <row r="15" ht="15" customHeight="1" s="15">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>Tools (IYA Makerspace)</t>
-        </is>
-      </c>
-      <c r="B15" s="21" t="n"/>
-      <c r="C15" s="21" t="n"/>
-      <c r="D15" s="21" t="n"/>
-      <c r="E15" s="21" t="n"/>
-      <c r="F15" s="21" t="n"/>
-      <c r="G15" s="21" t="n"/>
-      <c r="H15" s="21" t="n"/>
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Heat-shrink tubing</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>Covers the motor wire joints</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>Small (1–2 mm) heat-shrink</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>IYA Makerspace</t>
+        </is>
+      </c>
+      <c r="E15" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="25">
+        <f>E15*F15</f>
+        <v/>
+      </c>
+      <c r="H15" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="15">
-      <c r="A16" s="22" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="B16" s="22" t="inlineStr">
-        <is>
-          <t>What it is for</t>
-        </is>
-      </c>
-      <c r="C16" s="22" t="inlineStr">
-        <is>
-          <t>Exact part number</t>
-        </is>
-      </c>
-      <c r="D16" s="22" t="inlineStr">
-        <is>
-          <t>Buy from</t>
-        </is>
-      </c>
-      <c r="E16" s="22" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="F16" s="22" t="inlineStr">
-        <is>
-          <t>Price each</t>
-        </is>
-      </c>
-      <c r="G16" s="22" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="H16" s="22" t="inlineStr">
-        <is>
-          <t>Bought?</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="15">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Programmer</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="inlineStr">
-        <is>
-          <t>Puts our software on the board</t>
-        </is>
-      </c>
-      <c r="C17" s="19" t="inlineStr">
-        <is>
-          <t>Nordic nRF54L15-DK ($39 at Digi-Key if not borrowed)</t>
-        </is>
-      </c>
-      <c r="D17" s="19" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Multimeter</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>Check battery + / − and shorts</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>Any basic multimeter</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
         <is>
           <t>IYA Makerspace</t>
         </is>
       </c>
-      <c r="E17" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="24" t="n">
+      <c r="E16" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="G17" s="25">
-        <f>E17*F17</f>
+      <c r="G16" s="25">
+        <f>E16*F16</f>
         <v/>
       </c>
-      <c r="H17" s="26" t="inlineStr">
+      <c r="H16" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
+    <row r="17" s="15"/>
     <row r="18" ht="15" customHeight="1" s="15">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>Debug cable</t>
-        </is>
-      </c>
-      <c r="B18" s="19" t="inlineStr">
-        <is>
-          <t>Connects programmer to board</t>
-        </is>
-      </c>
-      <c r="C18" s="19" t="inlineStr">
-        <is>
-          <t>Samtec FFSD-05-D-02.00-01-N, 10-pin, 5 cm ($10.59 at Digi-Key)</t>
-        </is>
-      </c>
-      <c r="D18" s="19" t="inlineStr">
-        <is>
-          <t>IYA Makerspace</t>
-        </is>
-      </c>
-      <c r="E18" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="25">
-        <f>E18*F18</f>
+      <c r="F18" s="27" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="G18" s="28">
+        <f>SUMPRODUCT(E5:E17,F5:F17)</f>
         <v/>
       </c>
-      <c r="H18" s="26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="26.85" customHeight="1" s="15">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>Solder + flux</t>
-        </is>
-      </c>
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>To solder the module and buttons</t>
-        </is>
-      </c>
-      <c r="C19" s="19" t="inlineStr">
-        <is>
-          <t>Solder wire + no-clean flux</t>
-        </is>
-      </c>
-      <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>IYA Makerspace</t>
-        </is>
-      </c>
-      <c r="E19" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="25">
-        <f>E19*F19</f>
-        <v/>
-      </c>
-      <c r="H19" s="26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="15">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Heat-shrink tubing</t>
-        </is>
-      </c>
-      <c r="B20" s="19" t="inlineStr">
-        <is>
-          <t>Covers the motor wire joints</t>
-        </is>
-      </c>
-      <c r="C20" s="19" t="inlineStr">
-        <is>
-          <t>Small (1–2 mm) heat-shrink</t>
-        </is>
-      </c>
-      <c r="D20" s="19" t="inlineStr">
-        <is>
-          <t>IYA Makerspace</t>
-        </is>
-      </c>
-      <c r="E20" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="25">
-        <f>E20*F20</f>
-        <v/>
-      </c>
-      <c r="H20" s="26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="15">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Multimeter</t>
-        </is>
-      </c>
-      <c r="B21" s="19" t="inlineStr">
-        <is>
-          <t>Check battery + / − and shorts</t>
-        </is>
-      </c>
-      <c r="C21" s="19" t="inlineStr">
-        <is>
-          <t>Any basic multimeter</t>
-        </is>
-      </c>
-      <c r="D21" s="19" t="inlineStr">
-        <is>
-          <t>IYA Makerspace</t>
-        </is>
-      </c>
-      <c r="E21" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="25">
-        <f>E21*F21</f>
-        <v/>
-      </c>
-      <c r="H21" s="26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="15">
-      <c r="F23" s="27" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="G23" s="28">
-        <f>SUMPRODUCT(E5:E22,F5:F22)</f>
-        <v/>
-      </c>
-    </row>
+    </row>
+    <row r="19" s="15"/>
+    <row r="20" s="15"/>
+    <row r="21" s="15"/>
+    <row r="22" s="15"/>
+    <row r="23" s="15"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H6 H10:H13 H17:H21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="H5:H8 H12:H16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Dev board: the team solders the radio module on; JLCPCB fits the rest
Correction to the previous change: the 5 boards come assembled from JLCPCB with
everything except the radio module, which the team buys from Digi-Key and solders on.

- U1 is back out of fab/bom.csv and fab/cpl.csv; SW1 and SW2 stay in.
- README and parts_list.xlsx updated to match (6 modules: one per board plus a spare).

Gerbers, schematic and PCB are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/devboard/parts_list.xlsx
+++ b/hardware/devboard/parts_list.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="14" min="1" max="1"/>
@@ -801,75 +801,50 @@
     <row r="15" ht="15" customHeight="1" s="15">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t>Bluetooth module (pre-order it first)</t>
+          <t>Buttons</t>
         </is>
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>The brain + Bluetooth</t>
+          <t>Power and calibrate buttons</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>SW1, SW2</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>C45868630</t>
+          <t>C231329</t>
         </is>
       </c>
       <c r="E15" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" ht="52.2" customHeight="1" s="15">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t>Buttons</t>
+          <t>Small parts</t>
         </is>
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>Power and calibrate buttons</t>
+          <t>Resistors and capacitors (24 pieces)</t>
         </is>
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>SW1, SW2</t>
+          <t>C1,C4,C11,C12,C17,C19, C2,C5,C6,C18,C20,C21, C3, C16, C8,C9,C10,C22, R1,R2, R3, R6, R7,R8</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>C231329</t>
+          <t>see bom.csv</t>
         </is>
       </c>
       <c r="E16" s="19" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" ht="52.2" customHeight="1" s="15">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Small parts</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="inlineStr">
-        <is>
-          <t>Resistors and capacitors (24 pieces)</t>
-        </is>
-      </c>
-      <c r="C17" s="19" t="inlineStr">
-        <is>
-          <t>C1,C4,C11,C12,C17,C19, C2,C5,C6,C18,C20,C21, C3, C16, C8,C9,C10,C22, R1,R2, R3, R6, R7,R8</t>
-        </is>
-      </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>see bom.csv</t>
-        </is>
-      </c>
-      <c r="E17" s="19" t="n">
         <v>24</v>
       </c>
     </row>
@@ -886,7 +861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="14" min="1" max="1"/>
@@ -905,10 +880,11 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="15">
       <c r="A3" s="20" t="inlineStr">
         <is>
-          <t>Plugs into the board</t>
+          <t>On the board (we solder)</t>
         </is>
       </c>
       <c r="B3" s="21" t="n"/>
@@ -964,17 +940,17 @@
     <row r="5" ht="15" customHeight="1" s="15">
       <c r="A5" s="18" t="inlineStr">
         <is>
-          <t>Antenna</t>
+          <t>Bluetooth module</t>
         </is>
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>Bluetooth signal</t>
+          <t>The brain + Bluetooth</t>
         </is>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Taoglas FXP830.24.0100B (MHF4 plug)</t>
+          <t>Ezurio BL54L15 453-00044R</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -983,10 +959,10 @@
         </is>
       </c>
       <c r="E5" s="23" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F5" s="24" t="n">
-        <v>7.31</v>
+        <v>5.55</v>
       </c>
       <c r="G5" s="25">
         <f>E5*F5</f>
@@ -998,200 +974,200 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="15">
-      <c r="A6" s="18" t="inlineStr">
+    <row r="6" s="15"/>
+    <row r="7" ht="15" customHeight="1" s="15">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Plugs into the board</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="21" t="n"/>
+      <c r="G7" s="21" t="n"/>
+      <c r="H7" s="21" t="n"/>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="15">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>What it is for</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>Exact part number</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>Buy from</t>
+        </is>
+      </c>
+      <c r="E8" s="22" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="F8" s="22" t="inlineStr">
+        <is>
+          <t>Price each</t>
+        </is>
+      </c>
+      <c r="G8" s="22" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H8" s="22" t="inlineStr">
+        <is>
+          <t>Bought?</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="15">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Antenna</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Bluetooth signal</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>Taoglas FXP830.24.0100B (MHF4 plug)</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Digi-Key</t>
+        </is>
+      </c>
+      <c r="E9" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="24" t="n">
+        <v>7.31</v>
+      </c>
+      <c r="G9" s="25">
+        <f>E9*F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="15">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Battery</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>Power</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C10" s="19" t="inlineStr">
         <is>
           <t>Adafruit #1570 (100 mAh LiPo)</t>
         </is>
       </c>
-      <c r="D6" s="19" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>Adafruit</t>
         </is>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E10" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="24" t="n">
+      <c r="F10" s="24" t="n">
         <v>5.95</v>
       </c>
-      <c r="G6" s="25">
-        <f>E6*F6</f>
+      <c r="G10" s="25">
+        <f>E10*F10</f>
         <v/>
       </c>
-      <c r="H6" s="26" t="inlineStr">
+      <c r="H10" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="15">
-      <c r="A7" s="18" t="inlineStr">
+    <row r="11" ht="15" customHeight="1" s="15">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>Vibration motor</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>The "tap"</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C11" s="19" t="inlineStr">
         <is>
           <t>Vybronics VG0832022D</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>Digi-Key</t>
         </is>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E11" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="24" t="n">
+      <c r="F11" s="24" t="n">
         <v>3.47</v>
       </c>
-      <c r="G7" s="25">
-        <f>E7*F7</f>
+      <c r="G11" s="25">
+        <f>E11*F11</f>
         <v/>
       </c>
-      <c r="H7" s="26" t="inlineStr">
+      <c r="H11" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="26.85" customHeight="1" s="15">
-      <c r="A8" s="18" t="inlineStr">
+    <row r="12" ht="26.85" customHeight="1" s="15">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Motor cable</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
         <is>
           <t>Connects the motor to the board</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C12" s="19" t="inlineStr">
         <is>
           <t>JST SHR-02V-S housing + ASSHSSH28K102 lead, cut in half</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>Digi-Key</t>
         </is>
       </c>
-      <c r="E8" s="23" t="n">
+      <c r="E12" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="24" t="n">
+      <c r="F12" s="24" t="n">
         <v>0.6</v>
-      </c>
-      <c r="G8" s="25">
-        <f>E8*F8</f>
-        <v/>
-      </c>
-      <c r="H8" s="26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" s="15"/>
-    <row r="10" ht="15" customHeight="1" s="15">
-      <c r="A10" s="20" t="inlineStr">
-        <is>
-          <t>Tools (IYA Makerspace)</t>
-        </is>
-      </c>
-      <c r="B10" s="21" t="n"/>
-      <c r="C10" s="21" t="n"/>
-      <c r="D10" s="21" t="n"/>
-      <c r="E10" s="21" t="n"/>
-      <c r="F10" s="21" t="n"/>
-      <c r="G10" s="21" t="n"/>
-      <c r="H10" s="21" t="n"/>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="15">
-      <c r="A11" s="22" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="B11" s="22" t="inlineStr">
-        <is>
-          <t>What it is for</t>
-        </is>
-      </c>
-      <c r="C11" s="22" t="inlineStr">
-        <is>
-          <t>Exact part number</t>
-        </is>
-      </c>
-      <c r="D11" s="22" t="inlineStr">
-        <is>
-          <t>Buy from</t>
-        </is>
-      </c>
-      <c r="E11" s="22" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="F11" s="22" t="inlineStr">
-        <is>
-          <t>Price each</t>
-        </is>
-      </c>
-      <c r="G11" s="22" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="H11" s="22" t="inlineStr">
-        <is>
-          <t>Bought?</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="15">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Programmer</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>Puts our software on the board</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>Nordic nRF54L15-DK ($39 at Digi-Key if not borrowed)</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>IYA Makerspace</t>
-        </is>
-      </c>
-      <c r="E12" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="24" t="n">
-        <v>0</v>
       </c>
       <c r="G12" s="25">
         <f>E12*F12</f>
@@ -1203,131 +1179,77 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="15">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Debug cable</t>
-        </is>
-      </c>
-      <c r="B13" s="19" t="inlineStr">
-        <is>
-          <t>Connects programmer to board</t>
-        </is>
-      </c>
-      <c r="C13" s="19" t="inlineStr">
-        <is>
-          <t>Samtec FFSD-05-D-02.00-01-N, 10-pin, 5 cm ($10.59 at Digi-Key)</t>
-        </is>
-      </c>
-      <c r="D13" s="19" t="inlineStr">
-        <is>
-          <t>IYA Makerspace</t>
-        </is>
-      </c>
-      <c r="E13" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="25">
-        <f>E13*F13</f>
-        <v/>
-      </c>
-      <c r="H13" s="26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="26.85" customHeight="1" s="15">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Solder + flux</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>To join the motor wires to the motor cable</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>Solder wire + no-clean flux</t>
-        </is>
-      </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>IYA Makerspace</t>
-        </is>
-      </c>
-      <c r="E14" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="25">
-        <f>E14*F14</f>
-        <v/>
-      </c>
-      <c r="H14" s="26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+    <row r="13" s="15"/>
+    <row r="14" ht="15" customHeight="1" s="15">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>Tools (IYA Makerspace)</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="n"/>
+      <c r="C14" s="21" t="n"/>
+      <c r="D14" s="21" t="n"/>
+      <c r="E14" s="21" t="n"/>
+      <c r="F14" s="21" t="n"/>
+      <c r="G14" s="21" t="n"/>
+      <c r="H14" s="21" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="15">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Heat-shrink tubing</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>Covers the motor wire joints</t>
-        </is>
-      </c>
-      <c r="C15" s="19" t="inlineStr">
-        <is>
-          <t>Small (1–2 mm) heat-shrink</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>IYA Makerspace</t>
-        </is>
-      </c>
-      <c r="E15" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="25">
-        <f>E15*F15</f>
-        <v/>
-      </c>
-      <c r="H15" s="26" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>What it is for</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>Exact part number</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>Buy from</t>
+        </is>
+      </c>
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t>Price each</t>
+        </is>
+      </c>
+      <c r="G15" s="22" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H15" s="22" t="inlineStr">
+        <is>
+          <t>Bought?</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="15">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t>Multimeter</t>
+          <t>Programmer</t>
         </is>
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>Check battery + / − and shorts</t>
+          <t>Puts our software on the board</t>
         </is>
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>Any basic multimeter</t>
+          <t>Nordic nRF54L15-DK ($39 at Digi-Key if not borrowed)</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
@@ -1351,26 +1273,170 @@
         </is>
       </c>
     </row>
-    <row r="17" s="15"/>
-    <row r="18" ht="15" customHeight="1" s="15">
-      <c r="F18" s="27" t="inlineStr">
+    <row r="17" ht="15" customHeight="1" s="15">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Debug cable</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>Connects programmer to board</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>Samtec FFSD-05-D-02.00-01-N, 10-pin, 5 cm ($10.59 at Digi-Key)</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>IYA Makerspace</t>
+        </is>
+      </c>
+      <c r="E17" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="25">
+        <f>E17*F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26.85" customHeight="1" s="15">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Solder + flux</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>To solder the module and the motor wires</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>Solder wire + no-clean flux</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>IYA Makerspace</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="25">
+        <f>E18*F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="15">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>Heat-shrink tubing</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Covers the motor wire joints</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>Small (1–2 mm) heat-shrink</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>IYA Makerspace</t>
+        </is>
+      </c>
+      <c r="E19" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="25">
+        <f>E19*F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="15">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Multimeter</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>Check battery + / − and shorts</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>Any basic multimeter</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>IYA Makerspace</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="25">
+        <f>E20*F20</f>
+        <v/>
+      </c>
+      <c r="H20" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" s="15"/>
+    <row r="22" ht="15" customHeight="1" s="15">
+      <c r="F22" s="27" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="G18" s="28">
-        <f>SUMPRODUCT(E5:E17,F5:F17)</f>
+      <c r="G22" s="28">
+        <f>SUMPRODUCT(E5:E21,F5:F21)</f>
         <v/>
       </c>
     </row>
-    <row r="19" s="15"/>
-    <row r="20" s="15"/>
-    <row r="21" s="15"/>
-    <row r="22" s="15"/>
     <row r="23" s="15"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H8 H12:H16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H5 H9:H12 H16:H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>